<commit_message>
add John F Carter sette nadir
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/Sette.xlsx
+++ b/gu_in/Map.edf/Sette.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02675A6F-3404-4883-B02F-F7D2330DB7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEF521B-F905-4871-BBC6-9F49DAF7E448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5235" yWindow="1320" windowWidth="18480" windowHeight="11205" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="436">
   <si>
     <t>char[32]</t>
   </si>
@@ -1967,9 +1967,6 @@
     <t>settem32</t>
   </si>
   <si>
-    <t>dmm32_0</t>
-  </si>
-  <si>
     <t>sd141a3</t>
   </si>
   <si>
@@ -2136,6 +2133,15 @@
   </si>
   <si>
     <t>bd131B0</t>
+  </si>
+  <si>
+    <t>settem33</t>
+  </si>
+  <si>
+    <t>dmm33_0</t>
+  </si>
+  <si>
+    <t>17E17</t>
   </si>
 </sst>
 </file>
@@ -2193,9 +2199,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2536,7 +2543,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2986,7 +2993,7 @@
         <v>66</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D3" s="1">
         <v>46</v>
@@ -3072,7 +3079,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D4" s="1">
         <v>44</v>
@@ -3158,7 +3165,7 @@
         <v>66</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D5" s="1">
         <v>40</v>
@@ -3244,7 +3251,7 @@
         <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D6" s="1">
         <v>13</v>
@@ -3330,7 +3337,7 @@
         <v>77</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -3416,7 +3423,7 @@
         <v>77</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D8" s="1">
         <v>0</v>
@@ -3502,7 +3509,7 @@
         <v>68</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D9" s="1">
         <v>46</v>
@@ -3588,7 +3595,7 @@
         <v>68</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D10" s="1">
         <v>44</v>
@@ -3674,7 +3681,7 @@
         <v>68</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D11" s="1">
         <v>40</v>
@@ -3760,7 +3767,7 @@
         <v>68</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
@@ -3846,7 +3853,7 @@
         <v>68</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
@@ -4045,7 +4052,7 @@
         <v>203</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4062,7 +4069,7 @@
         <v>100</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -4079,7 +4086,7 @@
         <v>308</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4096,7 +4103,7 @@
         <v>308</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4113,7 +4120,7 @@
         <v>297</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4130,7 +4137,7 @@
         <v>249</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4147,7 +4154,7 @@
         <v>270</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4164,7 +4171,7 @@
         <v>241</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -4174,11 +4181,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J233"/>
+  <dimension ref="A1:J235"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -11070,7 +11080,7 @@
         <v>376</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>377</v>
+        <v>434</v>
       </c>
       <c r="C233" s="1">
         <v>25</v>
@@ -11094,6 +11104,52 @@
         <v>200</v>
       </c>
       <c r="J233" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10">
+      <c r="A234" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B234" s="1">
+        <v>0</v>
+      </c>
+      <c r="C234" s="1">
+        <v>0</v>
+      </c>
+      <c r="D234" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="1:10">
+      <c r="A235" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C235" s="1">
+        <v>25</v>
+      </c>
+      <c r="D235" s="1">
+        <v>0</v>
+      </c>
+      <c r="E235" s="1">
+        <v>-1957</v>
+      </c>
+      <c r="F235" s="1">
+        <v>-100</v>
+      </c>
+      <c r="G235" s="1">
+        <v>2454</v>
+      </c>
+      <c r="H235" s="1">
+        <v>100</v>
+      </c>
+      <c r="I235" s="1">
+        <v>200</v>
+      </c>
+      <c r="J235" s="1">
         <v>100</v>
       </c>
     </row>
@@ -11105,7 +11161,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="19.28515625" customWidth="1"/>
@@ -13266,6 +13322,32 @@
         <v>0</v>
       </c>
       <c r="H83" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="C84" s="1">
+        <v>28800000</v>
+      </c>
+      <c r="D84" s="1">
+        <v>1</v>
+      </c>
+      <c r="E84" s="1">
+        <v>100</v>
+      </c>
+      <c r="F84" s="1">
+        <v>0</v>
+      </c>
+      <c r="G84" s="1">
+        <v>0</v>
+      </c>
+      <c r="H84" s="1">
         <v>0</v>
       </c>
     </row>
@@ -14114,7 +14196,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B33" s="1">
         <v>315</v>
@@ -14140,7 +14222,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B34" s="1">
         <v>136</v>
@@ -14166,7 +14248,7 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B35" s="1">
         <v>35</v>
@@ -14192,7 +14274,7 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B36" s="1">
         <v>209</v>
@@ -14218,7 +14300,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B37" s="1">
         <v>0</v>
@@ -14244,7 +14326,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B38" s="1">
         <v>0</v>
@@ -14270,7 +14352,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B39" s="1">
         <v>144</v>
@@ -14296,7 +14378,7 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B40" s="1">
         <v>146</v>
@@ -14322,7 +14404,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B41" s="1">
         <v>146</v>
@@ -14348,7 +14430,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B42" s="1">
         <v>146</v>
@@ -14374,7 +14456,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B43" s="1">
         <v>0</v>
@@ -14400,7 +14482,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B44" s="1">
         <v>0</v>
@@ -14426,7 +14508,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B45" s="1">
         <v>0</v>
@@ -14452,7 +14534,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B46" s="1">
         <v>0</v>
@@ -14478,7 +14560,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B47" s="1">
         <v>0</v>
@@ -14504,7 +14586,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B48" s="1">
         <v>0</v>
@@ -14530,7 +14612,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B49" s="1">
         <v>0</v>
@@ -14556,7 +14638,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B50" s="1">
         <v>0</v>
@@ -14582,7 +14664,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B51" s="1">
         <v>0</v>
@@ -14608,7 +14690,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B52" s="1">
         <v>0</v>
@@ -14634,7 +14716,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B53" s="1">
         <v>0</v>
@@ -14660,7 +14742,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B54" s="1">
         <v>0</v>
@@ -14686,7 +14768,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B55" s="1">
         <v>0</v>
@@ -14712,7 +14794,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B56" s="1">
         <v>0</v>
@@ -14738,7 +14820,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B57" s="1">
         <v>0</v>
@@ -14764,7 +14846,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B58" s="1">
         <v>0</v>
@@ -14801,13 +14883,13 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -14824,22 +14906,22 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>403</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>404</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>96</v>
@@ -14865,7 +14947,7 @@
         <v>8</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -14888,7 +14970,7 @@
         <v>8</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -14911,7 +14993,7 @@
         <v>8</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -14934,7 +15016,7 @@
         <v>8</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -14957,7 +15039,7 @@
         <v>8</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -14980,7 +15062,7 @@
         <v>8</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -15003,7 +15085,7 @@
         <v>8</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Add John F Carter sette nadir map.edf
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/Sette.xlsx
+++ b/gu_in/Map.edf/Sette.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEF521B-F905-4871-BBC6-9F49DAF7E448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E96E47-A279-4616-931C-31A278C0CC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: Jetpack, kartert to golden pig, STC damage adjust, Chip HP adjust
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/Sette.xlsx
+++ b/gu_in/Map.edf/Sette.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project RF X\Parser_Public_Releases\Parser_official\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6827EDDF-5CAD-4301-A63C-0BE4474A7EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5316ED9E-0B73-42E6-A6A6-395ED729E724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="438">
   <si>
     <t>char[32]</t>
   </si>
@@ -2141,17 +2141,20 @@
     <t>dmm33_0</t>
   </si>
   <si>
-    <t>17E17</t>
-  </si>
-  <si>
     <t>dmm32_0</t>
+  </si>
+  <si>
+    <t>16407</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -2224,9 +2227,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2264,7 +2267,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2370,7 +2373,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2512,7 +2515,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2521,13 +2524,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2538,7 +2541,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2549,7 +2552,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -2560,7 +2563,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2571,7 +2574,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2604,7 +2607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -2615,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -2626,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -2637,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -2648,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -2659,7 +2662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
@@ -2670,7 +2673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
@@ -2681,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
@@ -2692,7 +2695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -2703,7 +2706,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -2714,7 +2717,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -2725,7 +2728,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
@@ -2736,7 +2739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -2747,7 +2750,7 @@
         <v>7475</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -2758,7 +2761,7 @@
         <v>7474</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -2769,7 +2772,7 @@
         <v>100782</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -2780,7 +2783,7 @@
         <v>108015</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -2800,7 +2803,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="2" width="27.7109375" customWidth="1"/>
@@ -2816,7 +2819,7 @@
     <col min="22" max="22" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2902,7 +2905,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:28">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -2988,7 +2991,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>65</v>
       </c>
@@ -3074,7 +3077,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>69</v>
       </c>
@@ -3160,7 +3163,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>71</v>
       </c>
@@ -3246,7 +3249,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>73</v>
       </c>
@@ -3332,7 +3335,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>76</v>
       </c>
@@ -3418,7 +3421,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>80</v>
       </c>
@@ -3504,7 +3507,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:28">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>68</v>
       </c>
@@ -3590,7 +3593,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>68</v>
       </c>
@@ -3676,7 +3679,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:28">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -3762,7 +3765,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:28">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>68</v>
       </c>
@@ -3848,7 +3851,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:28">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>68</v>
       </c>
@@ -3943,9 +3946,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -3971,7 +3974,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
@@ -4005,9 +4008,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -4024,7 +4027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>89</v>
       </c>
@@ -4041,7 +4044,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>51</v>
       </c>
@@ -4058,7 +4061,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>288</v>
       </c>
@@ -4075,7 +4078,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>72</v>
       </c>
@@ -4092,7 +4095,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>289</v>
       </c>
@@ -4109,7 +4112,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>112</v>
       </c>
@@ -4126,7 +4129,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>134</v>
       </c>
@@ -4143,7 +4146,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>280</v>
       </c>
@@ -4160,7 +4163,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>232</v>
       </c>
@@ -4185,7 +4188,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J235"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
@@ -4194,7 +4197,7 @@
     <col min="7" max="7" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -4226,7 +4229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -4258,7 +4261,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -4272,7 +4275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>107</v>
       </c>
@@ -4304,7 +4307,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>107</v>
       </c>
@@ -4336,7 +4339,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>107</v>
       </c>
@@ -4368,7 +4371,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>107</v>
       </c>
@@ -4400,7 +4403,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>115</v>
       </c>
@@ -4414,7 +4417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>115</v>
       </c>
@@ -4446,7 +4449,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>115</v>
       </c>
@@ -4478,7 +4481,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>115</v>
       </c>
@@ -4510,7 +4513,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>115</v>
       </c>
@@ -4542,7 +4545,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>123</v>
       </c>
@@ -4556,7 +4559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>123</v>
       </c>
@@ -4588,7 +4591,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>123</v>
       </c>
@@ -4620,7 +4623,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>123</v>
       </c>
@@ -4652,7 +4655,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>123</v>
       </c>
@@ -4684,7 +4687,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>128</v>
       </c>
@@ -4698,7 +4701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>128</v>
       </c>
@@ -4730,7 +4733,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>128</v>
       </c>
@@ -4762,7 +4765,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>128</v>
       </c>
@@ -4794,7 +4797,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>128</v>
       </c>
@@ -4826,7 +4829,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>138</v>
       </c>
@@ -4840,7 +4843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
@@ -4872,7 +4875,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>138</v>
       </c>
@@ -4904,7 +4907,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>138</v>
       </c>
@@ -4936,7 +4939,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>138</v>
       </c>
@@ -4968,7 +4971,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>144</v>
       </c>
@@ -4982,7 +4985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>144</v>
       </c>
@@ -5014,7 +5017,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>144</v>
       </c>
@@ -5046,7 +5049,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>144</v>
       </c>
@@ -5078,7 +5081,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>144</v>
       </c>
@@ -5110,7 +5113,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>149</v>
       </c>
@@ -5124,7 +5127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>149</v>
       </c>
@@ -5156,7 +5159,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>149</v>
       </c>
@@ -5188,7 +5191,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>149</v>
       </c>
@@ -5220,7 +5223,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>149</v>
       </c>
@@ -5252,7 +5255,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>158</v>
       </c>
@@ -5266,7 +5269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>158</v>
       </c>
@@ -5298,7 +5301,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>158</v>
       </c>
@@ -5330,7 +5333,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>158</v>
       </c>
@@ -5362,7 +5365,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>158</v>
       </c>
@@ -5394,7 +5397,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>163</v>
       </c>
@@ -5408,7 +5411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>163</v>
       </c>
@@ -5440,7 +5443,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>163</v>
       </c>
@@ -5472,7 +5475,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>163</v>
       </c>
@@ -5504,7 +5507,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>163</v>
       </c>
@@ -5536,7 +5539,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>169</v>
       </c>
@@ -5550,7 +5553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>169</v>
       </c>
@@ -5582,7 +5585,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>169</v>
       </c>
@@ -5614,7 +5617,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>169</v>
       </c>
@@ -5646,7 +5649,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>169</v>
       </c>
@@ -5678,7 +5681,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>169</v>
       </c>
@@ -5710,7 +5713,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>169</v>
       </c>
@@ -5742,7 +5745,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>169</v>
       </c>
@@ -5774,7 +5777,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>169</v>
       </c>
@@ -5806,7 +5809,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>169</v>
       </c>
@@ -5838,7 +5841,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>169</v>
       </c>
@@ -5870,7 +5873,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>169</v>
       </c>
@@ -5902,7 +5905,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>169</v>
       </c>
@@ -5934,7 +5937,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>169</v>
       </c>
@@ -5966,7 +5969,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>169</v>
       </c>
@@ -5998,7 +6001,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>169</v>
       </c>
@@ -6030,7 +6033,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>169</v>
       </c>
@@ -6062,7 +6065,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>187</v>
       </c>
@@ -6076,7 +6079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>187</v>
       </c>
@@ -6108,7 +6111,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>187</v>
       </c>
@@ -6140,7 +6143,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>187</v>
       </c>
@@ -6172,7 +6175,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>187</v>
       </c>
@@ -6204,7 +6207,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>187</v>
       </c>
@@ -6236,7 +6239,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>187</v>
       </c>
@@ -6268,7 +6271,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>187</v>
       </c>
@@ -6300,7 +6303,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>187</v>
       </c>
@@ -6332,7 +6335,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>187</v>
       </c>
@@ -6364,7 +6367,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>187</v>
       </c>
@@ -6396,7 +6399,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>187</v>
       </c>
@@ -6428,7 +6431,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>187</v>
       </c>
@@ -6460,7 +6463,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>187</v>
       </c>
@@ -6492,7 +6495,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>187</v>
       </c>
@@ -6524,7 +6527,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>187</v>
       </c>
@@ -6556,7 +6559,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>187</v>
       </c>
@@ -6588,7 +6591,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="1:10">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>204</v>
       </c>
@@ -6602,7 +6605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:10">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>204</v>
       </c>
@@ -6634,7 +6637,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:10">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>204</v>
       </c>
@@ -6666,7 +6669,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:10">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>204</v>
       </c>
@@ -6698,7 +6701,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="86" spans="1:10">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>204</v>
       </c>
@@ -6730,7 +6733,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="87" spans="1:10">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>204</v>
       </c>
@@ -6762,7 +6765,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="88" spans="1:10">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>204</v>
       </c>
@@ -6794,7 +6797,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="89" spans="1:10">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>204</v>
       </c>
@@ -6826,7 +6829,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="90" spans="1:10">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>204</v>
       </c>
@@ -6858,7 +6861,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>204</v>
       </c>
@@ -6890,7 +6893,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>204</v>
       </c>
@@ -6922,7 +6925,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>204</v>
       </c>
@@ -6954,7 +6957,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="94" spans="1:10">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>204</v>
       </c>
@@ -6986,7 +6989,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="95" spans="1:10">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>204</v>
       </c>
@@ -7018,7 +7021,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="96" spans="1:10">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>204</v>
       </c>
@@ -7050,7 +7053,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="97" spans="1:10">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>204</v>
       </c>
@@ -7082,7 +7085,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="98" spans="1:10">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>204</v>
       </c>
@@ -7114,7 +7117,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="99" spans="1:10">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>221</v>
       </c>
@@ -7128,7 +7131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>221</v>
       </c>
@@ -7160,7 +7163,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="101" spans="1:10">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>221</v>
       </c>
@@ -7192,7 +7195,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="102" spans="1:10">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>221</v>
       </c>
@@ -7224,7 +7227,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="103" spans="1:10">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>221</v>
       </c>
@@ -7256,7 +7259,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="104" spans="1:10">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>221</v>
       </c>
@@ -7288,7 +7291,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="105" spans="1:10">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>221</v>
       </c>
@@ -7320,7 +7323,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="106" spans="1:10">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>221</v>
       </c>
@@ -7352,7 +7355,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="107" spans="1:10">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>221</v>
       </c>
@@ -7384,7 +7387,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="108" spans="1:10">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>221</v>
       </c>
@@ -7416,7 +7419,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="109" spans="1:10">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>221</v>
       </c>
@@ -7448,7 +7451,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="110" spans="1:10">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>221</v>
       </c>
@@ -7480,7 +7483,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="111" spans="1:10">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>221</v>
       </c>
@@ -7512,7 +7515,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="112" spans="1:10">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>221</v>
       </c>
@@ -7544,7 +7547,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="113" spans="1:10">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>221</v>
       </c>
@@ -7576,7 +7579,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="114" spans="1:10">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>221</v>
       </c>
@@ -7608,7 +7611,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="115" spans="1:10">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>221</v>
       </c>
@@ -7640,7 +7643,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="116" spans="1:10">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>239</v>
       </c>
@@ -7654,7 +7657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:10">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>239</v>
       </c>
@@ -7686,7 +7689,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="118" spans="1:10">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>239</v>
       </c>
@@ -7718,7 +7721,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="119" spans="1:10">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>239</v>
       </c>
@@ -7750,7 +7753,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="120" spans="1:10">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>239</v>
       </c>
@@ -7782,7 +7785,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="121" spans="1:10">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>239</v>
       </c>
@@ -7814,7 +7817,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="122" spans="1:10">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>239</v>
       </c>
@@ -7846,7 +7849,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="123" spans="1:10">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>239</v>
       </c>
@@ -7878,7 +7881,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="124" spans="1:10">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>239</v>
       </c>
@@ -7910,7 +7913,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="125" spans="1:10">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>239</v>
       </c>
@@ -7942,7 +7945,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="126" spans="1:10">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>239</v>
       </c>
@@ -7974,7 +7977,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="127" spans="1:10">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>239</v>
       </c>
@@ -8006,7 +8009,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="128" spans="1:10">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>239</v>
       </c>
@@ -8038,7 +8041,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="129" spans="1:10">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>239</v>
       </c>
@@ -8070,7 +8073,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="130" spans="1:10">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>239</v>
       </c>
@@ -8102,7 +8105,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="131" spans="1:10">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>239</v>
       </c>
@@ -8134,7 +8137,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="132" spans="1:10">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>239</v>
       </c>
@@ -8166,7 +8169,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="133" spans="1:10">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>257</v>
       </c>
@@ -8180,7 +8183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:10">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>257</v>
       </c>
@@ -8212,7 +8215,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="135" spans="1:10">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>257</v>
       </c>
@@ -8244,7 +8247,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="136" spans="1:10">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>257</v>
       </c>
@@ -8276,7 +8279,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="137" spans="1:10">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>257</v>
       </c>
@@ -8308,7 +8311,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="138" spans="1:10">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>257</v>
       </c>
@@ -8340,7 +8343,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="139" spans="1:10">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>257</v>
       </c>
@@ -8372,7 +8375,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="140" spans="1:10">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>257</v>
       </c>
@@ -8404,7 +8407,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:10">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>257</v>
       </c>
@@ -8436,7 +8439,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="142" spans="1:10">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>257</v>
       </c>
@@ -8468,7 +8471,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="143" spans="1:10">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>257</v>
       </c>
@@ -8500,7 +8503,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:10">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>257</v>
       </c>
@@ -8532,7 +8535,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="145" spans="1:10">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>257</v>
       </c>
@@ -8564,7 +8567,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="146" spans="1:10">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>271</v>
       </c>
@@ -8578,7 +8581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:10">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>271</v>
       </c>
@@ -8610,7 +8613,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="148" spans="1:10">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>271</v>
       </c>
@@ -8642,7 +8645,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="149" spans="1:10">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>271</v>
       </c>
@@ -8674,7 +8677,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="150" spans="1:10">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>271</v>
       </c>
@@ -8706,7 +8709,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="151" spans="1:10">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>280</v>
       </c>
@@ -8720,7 +8723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:10">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>280</v>
       </c>
@@ -8752,7 +8755,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="153" spans="1:10">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>280</v>
       </c>
@@ -8784,7 +8787,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="154" spans="1:10">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>280</v>
       </c>
@@ -8816,7 +8819,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="155" spans="1:10">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>280</v>
       </c>
@@ -8848,7 +8851,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="156" spans="1:10">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>286</v>
       </c>
@@ -8862,7 +8865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:10">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>286</v>
       </c>
@@ -8894,7 +8897,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="158" spans="1:10">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>286</v>
       </c>
@@ -8926,7 +8929,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="159" spans="1:10">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>286</v>
       </c>
@@ -8958,7 +8961,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="160" spans="1:10">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>286</v>
       </c>
@@ -8990,7 +8993,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="161" spans="1:10">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>291</v>
       </c>
@@ -9004,7 +9007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:10">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>291</v>
       </c>
@@ -9036,7 +9039,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="163" spans="1:10">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>291</v>
       </c>
@@ -9068,7 +9071,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="164" spans="1:10">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>291</v>
       </c>
@@ -9100,7 +9103,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="165" spans="1:10">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>291</v>
       </c>
@@ -9132,7 +9135,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="166" spans="1:10">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>299</v>
       </c>
@@ -9146,7 +9149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:10">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>299</v>
       </c>
@@ -9178,7 +9181,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="168" spans="1:10">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>299</v>
       </c>
@@ -9210,7 +9213,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="169" spans="1:10">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>299</v>
       </c>
@@ -9242,7 +9245,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="170" spans="1:10">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>299</v>
       </c>
@@ -9274,7 +9277,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="171" spans="1:10">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>304</v>
       </c>
@@ -9288,7 +9291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:10">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>304</v>
       </c>
@@ -9320,7 +9323,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="173" spans="1:10">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>304</v>
       </c>
@@ -9352,7 +9355,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="174" spans="1:10">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>304</v>
       </c>
@@ -9384,7 +9387,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="175" spans="1:10">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>304</v>
       </c>
@@ -9416,7 +9419,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="176" spans="1:10">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>309</v>
       </c>
@@ -9430,7 +9433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:10">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>309</v>
       </c>
@@ -9462,7 +9465,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="178" spans="1:10">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>309</v>
       </c>
@@ -9494,7 +9497,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="179" spans="1:10">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>309</v>
       </c>
@@ -9526,7 +9529,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="180" spans="1:10">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>309</v>
       </c>
@@ -9558,7 +9561,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="181" spans="1:10">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>318</v>
       </c>
@@ -9572,7 +9575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:10">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>318</v>
       </c>
@@ -9604,7 +9607,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="183" spans="1:10">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>318</v>
       </c>
@@ -9636,7 +9639,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="184" spans="1:10">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>318</v>
       </c>
@@ -9668,7 +9671,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="185" spans="1:10">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>318</v>
       </c>
@@ -9700,7 +9703,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="186" spans="1:10">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>318</v>
       </c>
@@ -9732,7 +9735,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="187" spans="1:10">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>318</v>
       </c>
@@ -9764,7 +9767,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="188" spans="1:10">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>318</v>
       </c>
@@ -9796,7 +9799,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="189" spans="1:10">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>318</v>
       </c>
@@ -9828,7 +9831,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="190" spans="1:10">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>328</v>
       </c>
@@ -9842,7 +9845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:10">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>328</v>
       </c>
@@ -9874,7 +9877,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="192" spans="1:10">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>328</v>
       </c>
@@ -9906,7 +9909,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="193" spans="1:10">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>328</v>
       </c>
@@ -9938,7 +9941,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:10">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>328</v>
       </c>
@@ -9970,7 +9973,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="195" spans="1:10">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>328</v>
       </c>
@@ -10002,7 +10005,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="196" spans="1:10">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>328</v>
       </c>
@@ -10034,7 +10037,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="197" spans="1:10">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>328</v>
       </c>
@@ -10066,7 +10069,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="198" spans="1:10">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>328</v>
       </c>
@@ -10098,7 +10101,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="199" spans="1:10">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>328</v>
       </c>
@@ -10130,7 +10133,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="200" spans="1:10">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>328</v>
       </c>
@@ -10162,7 +10165,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="201" spans="1:10">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>328</v>
       </c>
@@ -10194,7 +10197,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="202" spans="1:10">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>328</v>
       </c>
@@ -10226,7 +10229,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="203" spans="1:10">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>328</v>
       </c>
@@ -10258,7 +10261,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="204" spans="1:10">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>328</v>
       </c>
@@ -10290,7 +10293,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="205" spans="1:10">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>328</v>
       </c>
@@ -10322,7 +10325,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="206" spans="1:10">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>328</v>
       </c>
@@ -10354,7 +10357,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="207" spans="1:10">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>346</v>
       </c>
@@ -10368,7 +10371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:10">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>346</v>
       </c>
@@ -10400,7 +10403,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="209" spans="1:10">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>346</v>
       </c>
@@ -10432,7 +10435,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="210" spans="1:10">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>346</v>
       </c>
@@ -10464,7 +10467,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="211" spans="1:10">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>346</v>
       </c>
@@ -10496,7 +10499,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="212" spans="1:10">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>352</v>
       </c>
@@ -10510,7 +10513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:10">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>352</v>
       </c>
@@ -10542,7 +10545,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="214" spans="1:10">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>352</v>
       </c>
@@ -10574,7 +10577,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="215" spans="1:10">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>352</v>
       </c>
@@ -10606,7 +10609,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="216" spans="1:10">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>352</v>
       </c>
@@ -10638,7 +10641,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="217" spans="1:10">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>358</v>
       </c>
@@ -10652,7 +10655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:10">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>358</v>
       </c>
@@ -10684,7 +10687,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="219" spans="1:10">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>358</v>
       </c>
@@ -10716,7 +10719,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="220" spans="1:10">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>358</v>
       </c>
@@ -10748,7 +10751,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="221" spans="1:10">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>358</v>
       </c>
@@ -10780,7 +10783,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="222" spans="1:10">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>364</v>
       </c>
@@ -10794,7 +10797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:10">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>364</v>
       </c>
@@ -10826,7 +10829,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="224" spans="1:10">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>364</v>
       </c>
@@ -10858,7 +10861,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="225" spans="1:10">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>364</v>
       </c>
@@ -10890,7 +10893,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="226" spans="1:10">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>364</v>
       </c>
@@ -10922,7 +10925,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="227" spans="1:10">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>370</v>
       </c>
@@ -10936,7 +10939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:10">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>370</v>
       </c>
@@ -10968,7 +10971,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="229" spans="1:10">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>370</v>
       </c>
@@ -11000,7 +11003,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="230" spans="1:10">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>370</v>
       </c>
@@ -11032,7 +11035,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="231" spans="1:10">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
         <v>370</v>
       </c>
@@ -11064,7 +11067,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="232" spans="1:10">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>376</v>
       </c>
@@ -11078,12 +11081,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:10">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>376</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C233" s="1">
         <v>25</v>
@@ -11110,7 +11113,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="234" spans="1:10">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>433</v>
       </c>
@@ -11124,7 +11127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:10">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>433</v>
       </c>
@@ -11164,13 +11167,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H84"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:K86"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -11196,7 +11199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -11222,7 +11225,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -11248,7 +11251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>107</v>
       </c>
@@ -11274,7 +11277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>107</v>
       </c>
@@ -11300,7 +11303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>115</v>
       </c>
@@ -11326,7 +11329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>115</v>
       </c>
@@ -11352,7 +11355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>115</v>
       </c>
@@ -11378,7 +11381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>115</v>
       </c>
@@ -11404,7 +11407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>123</v>
       </c>
@@ -11430,7 +11433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>123</v>
       </c>
@@ -11456,7 +11459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>123</v>
       </c>
@@ -11482,7 +11485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>123</v>
       </c>
@@ -11508,7 +11511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>123</v>
       </c>
@@ -11534,7 +11537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>128</v>
       </c>
@@ -11560,7 +11563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>128</v>
       </c>
@@ -11586,7 +11589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>128</v>
       </c>
@@ -11612,7 +11615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>128</v>
       </c>
@@ -11638,7 +11641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>128</v>
       </c>
@@ -11664,7 +11667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>138</v>
       </c>
@@ -11690,7 +11693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>138</v>
       </c>
@@ -11716,7 +11719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>138</v>
       </c>
@@ -11742,7 +11745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>138</v>
       </c>
@@ -11768,7 +11771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
@@ -11794,7 +11797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>144</v>
       </c>
@@ -11820,7 +11823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>144</v>
       </c>
@@ -11846,7 +11849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>144</v>
       </c>
@@ -11872,7 +11875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>144</v>
       </c>
@@ -11898,7 +11901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>149</v>
       </c>
@@ -11924,7 +11927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>149</v>
       </c>
@@ -11950,7 +11953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>149</v>
       </c>
@@ -11976,7 +11979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>149</v>
       </c>
@@ -12002,7 +12005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>158</v>
       </c>
@@ -12028,7 +12031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>158</v>
       </c>
@@ -12054,7 +12057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>158</v>
       </c>
@@ -12080,7 +12083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>158</v>
       </c>
@@ -12106,7 +12109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>163</v>
       </c>
@@ -12132,7 +12135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>163</v>
       </c>
@@ -12158,7 +12161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>163</v>
       </c>
@@ -12184,7 +12187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>163</v>
       </c>
@@ -12210,7 +12213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>169</v>
       </c>
@@ -12236,7 +12239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>187</v>
       </c>
@@ -12262,7 +12265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>204</v>
       </c>
@@ -12288,7 +12291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>221</v>
       </c>
@@ -12314,7 +12317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>239</v>
       </c>
@@ -12340,7 +12343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>257</v>
       </c>
@@ -12366,7 +12369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>271</v>
       </c>
@@ -12392,7 +12395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>271</v>
       </c>
@@ -12418,7 +12421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>271</v>
       </c>
@@ -12444,7 +12447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>271</v>
       </c>
@@ -12470,7 +12473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>280</v>
       </c>
@@ -12496,7 +12499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>280</v>
       </c>
@@ -12522,7 +12525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>280</v>
       </c>
@@ -12548,7 +12551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>280</v>
       </c>
@@ -12574,7 +12577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>280</v>
       </c>
@@ -12600,7 +12603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>286</v>
       </c>
@@ -12626,7 +12629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>286</v>
       </c>
@@ -12652,7 +12655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>286</v>
       </c>
@@ -12678,7 +12681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>286</v>
       </c>
@@ -12704,7 +12707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>291</v>
       </c>
@@ -12730,7 +12733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>291</v>
       </c>
@@ -12756,7 +12759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>291</v>
       </c>
@@ -12782,7 +12785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>299</v>
       </c>
@@ -12808,7 +12811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>299</v>
       </c>
@@ -12834,7 +12837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>299</v>
       </c>
@@ -12860,7 +12863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>304</v>
       </c>
@@ -12886,7 +12889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>304</v>
       </c>
@@ -12912,7 +12915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>304</v>
       </c>
@@ -12938,7 +12941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>309</v>
       </c>
@@ -12964,7 +12967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>309</v>
       </c>
@@ -12990,7 +12993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>309</v>
       </c>
@@ -13016,7 +13019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>309</v>
       </c>
@@ -13042,7 +13045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>318</v>
       </c>
@@ -13068,7 +13071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>318</v>
       </c>
@@ -13094,7 +13097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>318</v>
       </c>
@@ -13120,7 +13123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>318</v>
       </c>
@@ -13146,7 +13149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>328</v>
       </c>
@@ -13172,7 +13175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>346</v>
       </c>
@@ -13198,7 +13201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>352</v>
       </c>
@@ -13224,7 +13227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>358</v>
       </c>
@@ -13250,7 +13253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>364</v>
       </c>
@@ -13276,7 +13279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>370</v>
       </c>
@@ -13302,11 +13305,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B83" s="1">
+      <c r="B83" s="2">
         <v>23301</v>
       </c>
       <c r="C83" s="1">
@@ -13328,12 +13331,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>433</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C84" s="1">
         <v>28800000</v>
@@ -13352,6 +13355,11 @@
       </c>
       <c r="H84" s="1">
         <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K86" t="s">
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -13363,9 +13371,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H58"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -13391,7 +13399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -13417,7 +13425,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -13443,7 +13451,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>115</v>
       </c>
@@ -13469,7 +13477,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
@@ -13495,7 +13503,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>128</v>
       </c>
@@ -13521,7 +13529,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>138</v>
       </c>
@@ -13547,7 +13555,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>144</v>
       </c>
@@ -13573,7 +13581,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>149</v>
       </c>
@@ -13599,7 +13607,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>158</v>
       </c>
@@ -13625,7 +13633,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>163</v>
       </c>
@@ -13651,7 +13659,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>168</v>
       </c>
@@ -13677,7 +13685,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>169</v>
       </c>
@@ -13703,7 +13711,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>187</v>
       </c>
@@ -13729,7 +13737,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>204</v>
       </c>
@@ -13755,7 +13763,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>221</v>
       </c>
@@ -13781,7 +13789,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>239</v>
       </c>
@@ -13807,7 +13815,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>257</v>
       </c>
@@ -13833,7 +13841,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>271</v>
       </c>
@@ -13859,7 +13867,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>280</v>
       </c>
@@ -13885,7 +13893,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>286</v>
       </c>
@@ -13911,7 +13919,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>291</v>
       </c>
@@ -13937,7 +13945,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>299</v>
       </c>
@@ -13963,7 +13971,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>304</v>
       </c>
@@ -13989,7 +13997,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>309</v>
       </c>
@@ -14015,7 +14023,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>318</v>
       </c>
@@ -14041,7 +14049,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>328</v>
       </c>
@@ -14067,7 +14075,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>346</v>
       </c>
@@ -14093,7 +14101,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>352</v>
       </c>
@@ -14119,7 +14127,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>358</v>
       </c>
@@ -14145,7 +14153,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>364</v>
       </c>
@@ -14171,7 +14179,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>370</v>
       </c>
@@ -14197,7 +14205,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>377</v>
       </c>
@@ -14223,7 +14231,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>378</v>
       </c>
@@ -14249,7 +14257,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>379</v>
       </c>
@@ -14275,7 +14283,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>380</v>
       </c>
@@ -14301,7 +14309,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>381</v>
       </c>
@@ -14327,7 +14335,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>382</v>
       </c>
@@ -14353,7 +14361,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>383</v>
       </c>
@@ -14379,7 +14387,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>384</v>
       </c>
@@ -14405,7 +14413,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>385</v>
       </c>
@@ -14431,7 +14439,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>386</v>
       </c>
@@ -14457,7 +14465,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>387</v>
       </c>
@@ -14483,7 +14491,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>388</v>
       </c>
@@ -14509,7 +14517,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>389</v>
       </c>
@@ -14535,7 +14543,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>390</v>
       </c>
@@ -14561,7 +14569,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>391</v>
       </c>
@@ -14587,7 +14595,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>392</v>
       </c>
@@ -14613,7 +14621,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>393</v>
       </c>
@@ -14639,7 +14647,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>394</v>
       </c>
@@ -14665,7 +14673,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>395</v>
       </c>
@@ -14691,7 +14699,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>396</v>
       </c>
@@ -14717,7 +14725,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>427</v>
       </c>
@@ -14743,7 +14751,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>428</v>
       </c>
@@ -14769,7 +14777,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>429</v>
       </c>
@@ -14795,7 +14803,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>430</v>
       </c>
@@ -14821,7 +14829,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>431</v>
       </c>
@@ -14847,7 +14855,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>432</v>
       </c>
@@ -14882,9 +14890,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>397</v>
       </c>
@@ -14907,7 +14915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>398</v>
       </c>
@@ -14930,7 +14938,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -14953,7 +14961,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>51</v>
       </c>
@@ -14976,7 +14984,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>101</v>
       </c>
@@ -14999,7 +15007,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>151</v>
       </c>
@@ -15022,7 +15030,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>201</v>
       </c>
@@ -15045,7 +15053,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>251</v>
       </c>
@@ -15068,7 +15076,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
change Dark Loard to The Man
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/Sette.xlsx
+++ b/gu_in/Map.edf/Sette.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project RF X\Parser_Public_Releases\Parser_official\Database\gu_in\Map.edf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645925D9-5036-4DF0-8DAE-5E938ECF7ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7DD3AAB-EDD1-4B8F-888D-DF1214E5C4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="17565" windowHeight="11205" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="439">
   <si>
     <t>char[32]</t>
   </si>
@@ -2148,13 +2148,16 @@
   </si>
   <si>
     <t>16517</t>
+  </si>
+  <si>
+    <t>77E17</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -2173,7 +2176,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2183,6 +2186,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
       </patternFill>
     </fill>
   </fills>
@@ -2205,10 +2213,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2227,9 +2236,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2267,7 +2276,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2373,7 +2382,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2515,7 +2524,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2524,13 +2533,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2541,7 +2550,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2552,7 +2561,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -2563,7 +2572,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2574,7 +2583,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2585,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2596,7 +2605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2607,7 +2616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -2618,7 +2627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -2629,7 +2638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -2640,7 +2649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -2651,7 +2660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -2662,7 +2671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
@@ -2673,7 +2682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
@@ -2684,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
@@ -2695,7 +2704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -2706,7 +2715,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -2717,7 +2726,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -2728,7 +2737,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
@@ -2739,7 +2748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -2750,7 +2759,7 @@
         <v>7475</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -2761,7 +2770,7 @@
         <v>7474</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -2772,7 +2781,7 @@
         <v>100782</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -2783,7 +2792,7 @@
         <v>108015</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -2803,7 +2812,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="2" width="27.7109375" customWidth="1"/>
@@ -2819,7 +2828,7 @@
     <col min="22" max="22" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2905,7 +2914,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -2991,7 +3000,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28">
       <c r="A3" s="1" t="s">
         <v>65</v>
       </c>
@@ -3077,7 +3086,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28">
       <c r="A4" s="1" t="s">
         <v>69</v>
       </c>
@@ -3163,7 +3172,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28">
       <c r="A5" s="1" t="s">
         <v>71</v>
       </c>
@@ -3249,7 +3258,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28">
       <c r="A6" s="1" t="s">
         <v>73</v>
       </c>
@@ -3335,7 +3344,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28">
       <c r="A7" s="1" t="s">
         <v>76</v>
       </c>
@@ -3421,7 +3430,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28">
       <c r="A8" s="1" t="s">
         <v>80</v>
       </c>
@@ -3507,7 +3516,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28">
       <c r="A9" s="1" t="s">
         <v>68</v>
       </c>
@@ -3593,7 +3602,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28">
       <c r="A10" s="1" t="s">
         <v>68</v>
       </c>
@@ -3679,7 +3688,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -3765,7 +3774,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28">
       <c r="A12" s="1" t="s">
         <v>68</v>
       </c>
@@ -3851,7 +3860,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28">
       <c r="A13" s="1" t="s">
         <v>68</v>
       </c>
@@ -3946,9 +3955,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -3974,7 +3983,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
@@ -4008,9 +4017,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -4027,7 +4036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>89</v>
       </c>
@@ -4044,7 +4053,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="1">
         <v>51</v>
       </c>
@@ -4061,7 +4070,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" s="1">
         <v>288</v>
       </c>
@@ -4078,7 +4087,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" s="1">
         <v>72</v>
       </c>
@@ -4095,7 +4104,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" s="1">
         <v>289</v>
       </c>
@@ -4112,7 +4121,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" s="1">
         <v>112</v>
       </c>
@@ -4129,7 +4138,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" s="1">
         <v>134</v>
       </c>
@@ -4146,7 +4155,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" s="1">
         <v>280</v>
       </c>
@@ -4163,7 +4172,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" s="1">
         <v>232</v>
       </c>
@@ -4188,7 +4197,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J235"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
@@ -4197,7 +4206,7 @@
     <col min="7" max="7" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -4229,7 +4238,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -4261,7 +4270,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -4275,7 +4284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>107</v>
       </c>
@@ -4307,7 +4316,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
         <v>107</v>
       </c>
@@ -4339,7 +4348,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="A6" s="1" t="s">
         <v>107</v>
       </c>
@@ -4371,7 +4380,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="A7" s="1" t="s">
         <v>107</v>
       </c>
@@ -4403,7 +4412,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10">
       <c r="A8" s="1" t="s">
         <v>115</v>
       </c>
@@ -4417,7 +4426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="A9" s="1" t="s">
         <v>115</v>
       </c>
@@ -4449,7 +4458,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="A10" s="1" t="s">
         <v>115</v>
       </c>
@@ -4481,7 +4490,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="A11" s="1" t="s">
         <v>115</v>
       </c>
@@ -4513,7 +4522,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10">
       <c r="A12" s="1" t="s">
         <v>115</v>
       </c>
@@ -4545,7 +4554,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10">
       <c r="A13" s="1" t="s">
         <v>123</v>
       </c>
@@ -4559,7 +4568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10">
       <c r="A14" s="1" t="s">
         <v>123</v>
       </c>
@@ -4591,7 +4600,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10">
       <c r="A15" s="1" t="s">
         <v>123</v>
       </c>
@@ -4623,7 +4632,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="A16" s="1" t="s">
         <v>123</v>
       </c>
@@ -4655,7 +4664,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10">
       <c r="A17" s="1" t="s">
         <v>123</v>
       </c>
@@ -4687,7 +4696,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10">
       <c r="A18" s="1" t="s">
         <v>128</v>
       </c>
@@ -4701,7 +4710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10">
       <c r="A19" s="1" t="s">
         <v>128</v>
       </c>
@@ -4733,7 +4742,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
         <v>128</v>
       </c>
@@ -4765,7 +4774,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10">
       <c r="A21" s="1" t="s">
         <v>128</v>
       </c>
@@ -4797,7 +4806,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10">
       <c r="A22" s="1" t="s">
         <v>128</v>
       </c>
@@ -4829,7 +4838,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10">
       <c r="A23" s="1" t="s">
         <v>138</v>
       </c>
@@ -4843,7 +4852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10">
       <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
@@ -4875,7 +4884,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10">
       <c r="A25" s="1" t="s">
         <v>138</v>
       </c>
@@ -4907,7 +4916,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10">
       <c r="A26" s="1" t="s">
         <v>138</v>
       </c>
@@ -4939,7 +4948,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10">
       <c r="A27" s="1" t="s">
         <v>138</v>
       </c>
@@ -4971,7 +4980,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10">
       <c r="A28" s="1" t="s">
         <v>144</v>
       </c>
@@ -4985,7 +4994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10">
       <c r="A29" s="1" t="s">
         <v>144</v>
       </c>
@@ -5017,7 +5026,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10">
       <c r="A30" s="1" t="s">
         <v>144</v>
       </c>
@@ -5049,7 +5058,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
         <v>144</v>
       </c>
@@ -5081,7 +5090,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
         <v>144</v>
       </c>
@@ -5113,7 +5122,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10">
       <c r="A33" s="1" t="s">
         <v>149</v>
       </c>
@@ -5127,7 +5136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10">
       <c r="A34" s="1" t="s">
         <v>149</v>
       </c>
@@ -5159,7 +5168,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10">
       <c r="A35" s="1" t="s">
         <v>149</v>
       </c>
@@ -5191,7 +5200,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10">
       <c r="A36" s="1" t="s">
         <v>149</v>
       </c>
@@ -5223,7 +5232,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10">
       <c r="A37" s="1" t="s">
         <v>149</v>
       </c>
@@ -5255,7 +5264,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10">
       <c r="A38" s="1" t="s">
         <v>158</v>
       </c>
@@ -5269,7 +5278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10">
       <c r="A39" s="1" t="s">
         <v>158</v>
       </c>
@@ -5301,7 +5310,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10">
       <c r="A40" s="1" t="s">
         <v>158</v>
       </c>
@@ -5333,7 +5342,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10">
       <c r="A41" s="1" t="s">
         <v>158</v>
       </c>
@@ -5365,7 +5374,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10">
       <c r="A42" s="1" t="s">
         <v>158</v>
       </c>
@@ -5397,7 +5406,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10">
       <c r="A43" s="1" t="s">
         <v>163</v>
       </c>
@@ -5411,7 +5420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10">
       <c r="A44" s="1" t="s">
         <v>163</v>
       </c>
@@ -5443,7 +5452,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10">
       <c r="A45" s="1" t="s">
         <v>163</v>
       </c>
@@ -5475,7 +5484,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10">
       <c r="A46" s="1" t="s">
         <v>163</v>
       </c>
@@ -5507,7 +5516,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10">
       <c r="A47" s="1" t="s">
         <v>163</v>
       </c>
@@ -5539,7 +5548,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10">
       <c r="A48" s="1" t="s">
         <v>169</v>
       </c>
@@ -5553,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10">
       <c r="A49" s="1" t="s">
         <v>169</v>
       </c>
@@ -5585,7 +5594,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10">
       <c r="A50" s="1" t="s">
         <v>169</v>
       </c>
@@ -5617,7 +5626,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10">
       <c r="A51" s="1" t="s">
         <v>169</v>
       </c>
@@ -5649,7 +5658,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10">
       <c r="A52" s="1" t="s">
         <v>169</v>
       </c>
@@ -5681,7 +5690,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10">
       <c r="A53" s="1" t="s">
         <v>169</v>
       </c>
@@ -5713,7 +5722,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10">
       <c r="A54" s="1" t="s">
         <v>169</v>
       </c>
@@ -5745,7 +5754,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10">
       <c r="A55" s="1" t="s">
         <v>169</v>
       </c>
@@ -5777,7 +5786,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10">
       <c r="A56" s="1" t="s">
         <v>169</v>
       </c>
@@ -5809,7 +5818,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10">
       <c r="A57" s="1" t="s">
         <v>169</v>
       </c>
@@ -5841,7 +5850,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10">
       <c r="A58" s="1" t="s">
         <v>169</v>
       </c>
@@ -5873,7 +5882,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10">
       <c r="A59" s="1" t="s">
         <v>169</v>
       </c>
@@ -5905,7 +5914,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10">
       <c r="A60" s="1" t="s">
         <v>169</v>
       </c>
@@ -5937,7 +5946,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10">
       <c r="A61" s="1" t="s">
         <v>169</v>
       </c>
@@ -5969,7 +5978,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10">
       <c r="A62" s="1" t="s">
         <v>169</v>
       </c>
@@ -6001,7 +6010,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10">
       <c r="A63" s="1" t="s">
         <v>169</v>
       </c>
@@ -6033,7 +6042,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10">
       <c r="A64" s="1" t="s">
         <v>169</v>
       </c>
@@ -6065,7 +6074,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10">
       <c r="A65" s="1" t="s">
         <v>187</v>
       </c>
@@ -6079,7 +6088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10">
       <c r="A66" s="1" t="s">
         <v>187</v>
       </c>
@@ -6111,7 +6120,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10">
       <c r="A67" s="1" t="s">
         <v>187</v>
       </c>
@@ -6143,7 +6152,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10">
       <c r="A68" s="1" t="s">
         <v>187</v>
       </c>
@@ -6175,7 +6184,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10">
       <c r="A69" s="1" t="s">
         <v>187</v>
       </c>
@@ -6207,7 +6216,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10">
       <c r="A70" s="1" t="s">
         <v>187</v>
       </c>
@@ -6239,7 +6248,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10">
       <c r="A71" s="1" t="s">
         <v>187</v>
       </c>
@@ -6271,7 +6280,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10">
       <c r="A72" s="1" t="s">
         <v>187</v>
       </c>
@@ -6303,7 +6312,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10">
       <c r="A73" s="1" t="s">
         <v>187</v>
       </c>
@@ -6335,7 +6344,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10">
       <c r="A74" s="1" t="s">
         <v>187</v>
       </c>
@@ -6367,7 +6376,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10">
       <c r="A75" s="1" t="s">
         <v>187</v>
       </c>
@@ -6399,7 +6408,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10">
       <c r="A76" s="1" t="s">
         <v>187</v>
       </c>
@@ -6431,7 +6440,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10">
       <c r="A77" s="1" t="s">
         <v>187</v>
       </c>
@@ -6463,7 +6472,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10">
       <c r="A78" s="1" t="s">
         <v>187</v>
       </c>
@@ -6495,7 +6504,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10">
       <c r="A79" s="1" t="s">
         <v>187</v>
       </c>
@@ -6527,7 +6536,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10">
       <c r="A80" s="1" t="s">
         <v>187</v>
       </c>
@@ -6559,7 +6568,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10">
       <c r="A81" s="1" t="s">
         <v>187</v>
       </c>
@@ -6591,7 +6600,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10">
       <c r="A82" s="1" t="s">
         <v>204</v>
       </c>
@@ -6605,7 +6614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10">
       <c r="A83" s="1" t="s">
         <v>204</v>
       </c>
@@ -6637,7 +6646,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10">
       <c r="A84" s="1" t="s">
         <v>204</v>
       </c>
@@ -6669,7 +6678,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10">
       <c r="A85" s="1" t="s">
         <v>204</v>
       </c>
@@ -6701,7 +6710,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10">
       <c r="A86" s="1" t="s">
         <v>204</v>
       </c>
@@ -6733,7 +6742,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10">
       <c r="A87" s="1" t="s">
         <v>204</v>
       </c>
@@ -6765,7 +6774,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10">
       <c r="A88" s="1" t="s">
         <v>204</v>
       </c>
@@ -6797,7 +6806,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10">
       <c r="A89" s="1" t="s">
         <v>204</v>
       </c>
@@ -6829,7 +6838,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10">
       <c r="A90" s="1" t="s">
         <v>204</v>
       </c>
@@ -6861,7 +6870,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10">
       <c r="A91" s="1" t="s">
         <v>204</v>
       </c>
@@ -6893,7 +6902,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10">
       <c r="A92" s="1" t="s">
         <v>204</v>
       </c>
@@ -6925,7 +6934,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10">
       <c r="A93" s="1" t="s">
         <v>204</v>
       </c>
@@ -6957,7 +6966,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10">
       <c r="A94" s="1" t="s">
         <v>204</v>
       </c>
@@ -6989,7 +6998,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10">
       <c r="A95" s="1" t="s">
         <v>204</v>
       </c>
@@ -7021,7 +7030,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10">
       <c r="A96" s="1" t="s">
         <v>204</v>
       </c>
@@ -7053,7 +7062,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10">
       <c r="A97" s="1" t="s">
         <v>204</v>
       </c>
@@ -7085,7 +7094,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10">
       <c r="A98" s="1" t="s">
         <v>204</v>
       </c>
@@ -7117,7 +7126,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10">
       <c r="A99" s="1" t="s">
         <v>221</v>
       </c>
@@ -7131,7 +7140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10">
       <c r="A100" s="1" t="s">
         <v>221</v>
       </c>
@@ -7163,7 +7172,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10">
       <c r="A101" s="1" t="s">
         <v>221</v>
       </c>
@@ -7195,7 +7204,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10">
       <c r="A102" s="1" t="s">
         <v>221</v>
       </c>
@@ -7227,7 +7236,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10">
       <c r="A103" s="1" t="s">
         <v>221</v>
       </c>
@@ -7259,7 +7268,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10">
       <c r="A104" s="1" t="s">
         <v>221</v>
       </c>
@@ -7291,7 +7300,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10">
       <c r="A105" s="1" t="s">
         <v>221</v>
       </c>
@@ -7323,7 +7332,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10">
       <c r="A106" s="1" t="s">
         <v>221</v>
       </c>
@@ -7355,7 +7364,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10">
       <c r="A107" s="1" t="s">
         <v>221</v>
       </c>
@@ -7387,7 +7396,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10">
       <c r="A108" s="1" t="s">
         <v>221</v>
       </c>
@@ -7419,7 +7428,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10">
       <c r="A109" s="1" t="s">
         <v>221</v>
       </c>
@@ -7451,7 +7460,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10">
       <c r="A110" s="1" t="s">
         <v>221</v>
       </c>
@@ -7483,7 +7492,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10">
       <c r="A111" s="1" t="s">
         <v>221</v>
       </c>
@@ -7515,7 +7524,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10">
       <c r="A112" s="1" t="s">
         <v>221</v>
       </c>
@@ -7547,7 +7556,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10">
       <c r="A113" s="1" t="s">
         <v>221</v>
       </c>
@@ -7579,7 +7588,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10">
       <c r="A114" s="1" t="s">
         <v>221</v>
       </c>
@@ -7611,7 +7620,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10">
       <c r="A115" s="1" t="s">
         <v>221</v>
       </c>
@@ -7643,7 +7652,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10">
       <c r="A116" s="1" t="s">
         <v>239</v>
       </c>
@@ -7657,7 +7666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10">
       <c r="A117" s="1" t="s">
         <v>239</v>
       </c>
@@ -7689,7 +7698,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10">
       <c r="A118" s="1" t="s">
         <v>239</v>
       </c>
@@ -7721,7 +7730,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10">
       <c r="A119" s="1" t="s">
         <v>239</v>
       </c>
@@ -7753,7 +7762,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10">
       <c r="A120" s="1" t="s">
         <v>239</v>
       </c>
@@ -7785,7 +7794,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10">
       <c r="A121" s="1" t="s">
         <v>239</v>
       </c>
@@ -7817,7 +7826,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10">
       <c r="A122" s="1" t="s">
         <v>239</v>
       </c>
@@ -7849,7 +7858,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10">
       <c r="A123" s="1" t="s">
         <v>239</v>
       </c>
@@ -7881,7 +7890,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10">
       <c r="A124" s="1" t="s">
         <v>239</v>
       </c>
@@ -7913,7 +7922,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10">
       <c r="A125" s="1" t="s">
         <v>239</v>
       </c>
@@ -7945,7 +7954,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10">
       <c r="A126" s="1" t="s">
         <v>239</v>
       </c>
@@ -7977,7 +7986,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10">
       <c r="A127" s="1" t="s">
         <v>239</v>
       </c>
@@ -8009,7 +8018,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10">
       <c r="A128" s="1" t="s">
         <v>239</v>
       </c>
@@ -8041,7 +8050,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10">
       <c r="A129" s="1" t="s">
         <v>239</v>
       </c>
@@ -8073,7 +8082,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10">
       <c r="A130" s="1" t="s">
         <v>239</v>
       </c>
@@ -8105,7 +8114,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10">
       <c r="A131" s="1" t="s">
         <v>239</v>
       </c>
@@ -8137,7 +8146,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10">
       <c r="A132" s="1" t="s">
         <v>239</v>
       </c>
@@ -8169,7 +8178,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10">
       <c r="A133" s="1" t="s">
         <v>257</v>
       </c>
@@ -8183,7 +8192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10">
       <c r="A134" s="1" t="s">
         <v>257</v>
       </c>
@@ -8215,7 +8224,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10">
       <c r="A135" s="1" t="s">
         <v>257</v>
       </c>
@@ -8247,7 +8256,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10">
       <c r="A136" s="1" t="s">
         <v>257</v>
       </c>
@@ -8279,7 +8288,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10">
       <c r="A137" s="1" t="s">
         <v>257</v>
       </c>
@@ -8311,7 +8320,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10">
       <c r="A138" s="1" t="s">
         <v>257</v>
       </c>
@@ -8343,7 +8352,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10">
       <c r="A139" s="1" t="s">
         <v>257</v>
       </c>
@@ -8375,7 +8384,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10">
       <c r="A140" s="1" t="s">
         <v>257</v>
       </c>
@@ -8407,7 +8416,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10">
       <c r="A141" s="1" t="s">
         <v>257</v>
       </c>
@@ -8439,7 +8448,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10">
       <c r="A142" s="1" t="s">
         <v>257</v>
       </c>
@@ -8471,7 +8480,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10">
       <c r="A143" s="1" t="s">
         <v>257</v>
       </c>
@@ -8503,7 +8512,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10">
       <c r="A144" s="1" t="s">
         <v>257</v>
       </c>
@@ -8535,7 +8544,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10">
       <c r="A145" s="1" t="s">
         <v>257</v>
       </c>
@@ -8567,7 +8576,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10">
       <c r="A146" s="1" t="s">
         <v>271</v>
       </c>
@@ -8581,7 +8590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10">
       <c r="A147" s="1" t="s">
         <v>271</v>
       </c>
@@ -8613,7 +8622,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10">
       <c r="A148" s="1" t="s">
         <v>271</v>
       </c>
@@ -8645,7 +8654,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10">
       <c r="A149" s="1" t="s">
         <v>271</v>
       </c>
@@ -8677,7 +8686,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10">
       <c r="A150" s="1" t="s">
         <v>271</v>
       </c>
@@ -8709,7 +8718,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10">
       <c r="A151" s="1" t="s">
         <v>280</v>
       </c>
@@ -8723,7 +8732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10">
       <c r="A152" s="1" t="s">
         <v>280</v>
       </c>
@@ -8755,7 +8764,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10">
       <c r="A153" s="1" t="s">
         <v>280</v>
       </c>
@@ -8787,7 +8796,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10">
       <c r="A154" s="1" t="s">
         <v>280</v>
       </c>
@@ -8819,7 +8828,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10">
       <c r="A155" s="1" t="s">
         <v>280</v>
       </c>
@@ -8851,7 +8860,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10">
       <c r="A156" s="1" t="s">
         <v>286</v>
       </c>
@@ -8865,7 +8874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10">
       <c r="A157" s="1" t="s">
         <v>286</v>
       </c>
@@ -8897,7 +8906,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10">
       <c r="A158" s="1" t="s">
         <v>286</v>
       </c>
@@ -8929,7 +8938,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:10">
       <c r="A159" s="1" t="s">
         <v>286</v>
       </c>
@@ -8961,7 +8970,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10">
       <c r="A160" s="1" t="s">
         <v>286</v>
       </c>
@@ -8993,7 +9002,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10">
       <c r="A161" s="1" t="s">
         <v>291</v>
       </c>
@@ -9007,7 +9016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10">
       <c r="A162" s="1" t="s">
         <v>291</v>
       </c>
@@ -9039,7 +9048,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10">
       <c r="A163" s="1" t="s">
         <v>291</v>
       </c>
@@ -9071,7 +9080,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10">
       <c r="A164" s="1" t="s">
         <v>291</v>
       </c>
@@ -9103,7 +9112,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10">
       <c r="A165" s="1" t="s">
         <v>291</v>
       </c>
@@ -9135,7 +9144,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10">
       <c r="A166" s="1" t="s">
         <v>299</v>
       </c>
@@ -9149,7 +9158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:10">
       <c r="A167" s="1" t="s">
         <v>299</v>
       </c>
@@ -9181,7 +9190,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10">
       <c r="A168" s="1" t="s">
         <v>299</v>
       </c>
@@ -9213,7 +9222,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:10">
       <c r="A169" s="1" t="s">
         <v>299</v>
       </c>
@@ -9245,7 +9254,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10">
       <c r="A170" s="1" t="s">
         <v>299</v>
       </c>
@@ -9277,7 +9286,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10">
       <c r="A171" s="1" t="s">
         <v>304</v>
       </c>
@@ -9291,7 +9300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10">
       <c r="A172" s="1" t="s">
         <v>304</v>
       </c>
@@ -9323,7 +9332,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10">
       <c r="A173" s="1" t="s">
         <v>304</v>
       </c>
@@ -9355,7 +9364,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10">
       <c r="A174" s="1" t="s">
         <v>304</v>
       </c>
@@ -9387,7 +9396,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:10">
       <c r="A175" s="1" t="s">
         <v>304</v>
       </c>
@@ -9419,7 +9428,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:10">
       <c r="A176" s="1" t="s">
         <v>309</v>
       </c>
@@ -9433,7 +9442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:10">
       <c r="A177" s="1" t="s">
         <v>309</v>
       </c>
@@ -9465,7 +9474,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:10">
       <c r="A178" s="1" t="s">
         <v>309</v>
       </c>
@@ -9497,7 +9506,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:10">
       <c r="A179" s="1" t="s">
         <v>309</v>
       </c>
@@ -9529,7 +9538,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:10">
       <c r="A180" s="1" t="s">
         <v>309</v>
       </c>
@@ -9561,7 +9570,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:10">
       <c r="A181" s="1" t="s">
         <v>318</v>
       </c>
@@ -9575,7 +9584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:10">
       <c r="A182" s="1" t="s">
         <v>318</v>
       </c>
@@ -9607,7 +9616,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:10">
       <c r="A183" s="1" t="s">
         <v>318</v>
       </c>
@@ -9639,7 +9648,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:10">
       <c r="A184" s="1" t="s">
         <v>318</v>
       </c>
@@ -9671,7 +9680,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:10">
       <c r="A185" s="1" t="s">
         <v>318</v>
       </c>
@@ -9703,7 +9712,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:10">
       <c r="A186" s="1" t="s">
         <v>318</v>
       </c>
@@ -9735,7 +9744,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:10">
       <c r="A187" s="1" t="s">
         <v>318</v>
       </c>
@@ -9767,7 +9776,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:10">
       <c r="A188" s="1" t="s">
         <v>318</v>
       </c>
@@ -9799,7 +9808,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:10">
       <c r="A189" s="1" t="s">
         <v>318</v>
       </c>
@@ -9831,7 +9840,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:10">
       <c r="A190" s="1" t="s">
         <v>328</v>
       </c>
@@ -9845,7 +9854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:10">
       <c r="A191" s="1" t="s">
         <v>328</v>
       </c>
@@ -9877,7 +9886,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:10">
       <c r="A192" s="1" t="s">
         <v>328</v>
       </c>
@@ -9909,7 +9918,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:10">
       <c r="A193" s="1" t="s">
         <v>328</v>
       </c>
@@ -9941,7 +9950,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:10">
       <c r="A194" s="1" t="s">
         <v>328</v>
       </c>
@@ -9973,7 +9982,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:10">
       <c r="A195" s="1" t="s">
         <v>328</v>
       </c>
@@ -10005,7 +10014,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:10">
       <c r="A196" s="1" t="s">
         <v>328</v>
       </c>
@@ -10037,7 +10046,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:10">
       <c r="A197" s="1" t="s">
         <v>328</v>
       </c>
@@ -10069,7 +10078,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:10">
       <c r="A198" s="1" t="s">
         <v>328</v>
       </c>
@@ -10101,7 +10110,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:10">
       <c r="A199" s="1" t="s">
         <v>328</v>
       </c>
@@ -10133,7 +10142,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:10">
       <c r="A200" s="1" t="s">
         <v>328</v>
       </c>
@@ -10165,7 +10174,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:10">
       <c r="A201" s="1" t="s">
         <v>328</v>
       </c>
@@ -10197,7 +10206,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:10">
       <c r="A202" s="1" t="s">
         <v>328</v>
       </c>
@@ -10229,7 +10238,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:10">
       <c r="A203" s="1" t="s">
         <v>328</v>
       </c>
@@ -10261,7 +10270,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:10">
       <c r="A204" s="1" t="s">
         <v>328</v>
       </c>
@@ -10293,7 +10302,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:10">
       <c r="A205" s="1" t="s">
         <v>328</v>
       </c>
@@ -10325,7 +10334,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:10">
       <c r="A206" s="1" t="s">
         <v>328</v>
       </c>
@@ -10357,7 +10366,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:10">
       <c r="A207" s="1" t="s">
         <v>346</v>
       </c>
@@ -10371,7 +10380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:10">
       <c r="A208" s="1" t="s">
         <v>346</v>
       </c>
@@ -10403,7 +10412,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:10">
       <c r="A209" s="1" t="s">
         <v>346</v>
       </c>
@@ -10435,7 +10444,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:10">
       <c r="A210" s="1" t="s">
         <v>346</v>
       </c>
@@ -10467,7 +10476,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:10">
       <c r="A211" s="1" t="s">
         <v>346</v>
       </c>
@@ -10499,7 +10508,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:10">
       <c r="A212" s="1" t="s">
         <v>352</v>
       </c>
@@ -10513,7 +10522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:10">
       <c r="A213" s="1" t="s">
         <v>352</v>
       </c>
@@ -10545,7 +10554,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:10">
       <c r="A214" s="1" t="s">
         <v>352</v>
       </c>
@@ -10577,7 +10586,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:10">
       <c r="A215" s="1" t="s">
         <v>352</v>
       </c>
@@ -10609,7 +10618,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:10">
       <c r="A216" s="1" t="s">
         <v>352</v>
       </c>
@@ -10641,7 +10650,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:10">
       <c r="A217" s="1" t="s">
         <v>358</v>
       </c>
@@ -10655,7 +10664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:10">
       <c r="A218" s="1" t="s">
         <v>358</v>
       </c>
@@ -10687,7 +10696,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:10">
       <c r="A219" s="1" t="s">
         <v>358</v>
       </c>
@@ -10719,7 +10728,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:10">
       <c r="A220" s="1" t="s">
         <v>358</v>
       </c>
@@ -10751,7 +10760,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:10">
       <c r="A221" s="1" t="s">
         <v>358</v>
       </c>
@@ -10783,7 +10792,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:10">
       <c r="A222" s="1" t="s">
         <v>364</v>
       </c>
@@ -10797,7 +10806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:10">
       <c r="A223" s="1" t="s">
         <v>364</v>
       </c>
@@ -10829,7 +10838,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:10">
       <c r="A224" s="1" t="s">
         <v>364</v>
       </c>
@@ -10861,7 +10870,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:10">
       <c r="A225" s="1" t="s">
         <v>364</v>
       </c>
@@ -10893,7 +10902,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:10">
       <c r="A226" s="1" t="s">
         <v>364</v>
       </c>
@@ -10925,7 +10934,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:10">
       <c r="A227" s="1" t="s">
         <v>370</v>
       </c>
@@ -10939,7 +10948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:10">
       <c r="A228" s="1" t="s">
         <v>370</v>
       </c>
@@ -10971,7 +10980,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:10">
       <c r="A229" s="1" t="s">
         <v>370</v>
       </c>
@@ -11003,7 +11012,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:10">
       <c r="A230" s="1" t="s">
         <v>370</v>
       </c>
@@ -11035,7 +11044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:10">
       <c r="A231" s="1" t="s">
         <v>370</v>
       </c>
@@ -11067,7 +11076,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:10">
       <c r="A232" s="1" t="s">
         <v>376</v>
       </c>
@@ -11081,7 +11090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:10">
       <c r="A233" s="1" t="s">
         <v>376</v>
       </c>
@@ -11113,7 +11122,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:10">
       <c r="A234" s="1" t="s">
         <v>433</v>
       </c>
@@ -11127,7 +11136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:10">
       <c r="A235" s="1" t="s">
         <v>433</v>
       </c>
@@ -11168,12 +11177,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K86"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -11199,7 +11208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -11225,7 +11234,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -11251,7 +11260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>107</v>
       </c>
@@ -11277,7 +11286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
         <v>107</v>
       </c>
@@ -11303,7 +11312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
         <v>115</v>
       </c>
@@ -11329,7 +11338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
         <v>115</v>
       </c>
@@ -11355,7 +11364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
         <v>115</v>
       </c>
@@ -11381,7 +11390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
         <v>115</v>
       </c>
@@ -11407,7 +11416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
         <v>123</v>
       </c>
@@ -11433,7 +11442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="1" t="s">
         <v>123</v>
       </c>
@@ -11459,7 +11468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8">
       <c r="A12" s="1" t="s">
         <v>123</v>
       </c>
@@ -11485,7 +11494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8">
       <c r="A13" s="1" t="s">
         <v>123</v>
       </c>
@@ -11511,7 +11520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="1" t="s">
         <v>123</v>
       </c>
@@ -11537,7 +11546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8">
       <c r="A15" s="1" t="s">
         <v>128</v>
       </c>
@@ -11563,7 +11572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8">
       <c r="A16" s="1" t="s">
         <v>128</v>
       </c>
@@ -11589,7 +11598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="1" t="s">
         <v>128</v>
       </c>
@@ -11615,7 +11624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="1" t="s">
         <v>128</v>
       </c>
@@ -11641,7 +11650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
         <v>128</v>
       </c>
@@ -11667,7 +11676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="1" t="s">
         <v>138</v>
       </c>
@@ -11693,7 +11702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>138</v>
       </c>
@@ -11719,7 +11728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="1" t="s">
         <v>138</v>
       </c>
@@ -11745,7 +11754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8">
       <c r="A23" s="1" t="s">
         <v>138</v>
       </c>
@@ -11771,7 +11780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8">
       <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
@@ -11797,7 +11806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8">
       <c r="A25" s="1" t="s">
         <v>144</v>
       </c>
@@ -11823,7 +11832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8">
       <c r="A26" s="1" t="s">
         <v>144</v>
       </c>
@@ -11849,7 +11858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8">
       <c r="A27" s="1" t="s">
         <v>144</v>
       </c>
@@ -11875,7 +11884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8">
       <c r="A28" s="1" t="s">
         <v>144</v>
       </c>
@@ -11901,7 +11910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8">
       <c r="A29" s="1" t="s">
         <v>149</v>
       </c>
@@ -11927,7 +11936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8">
       <c r="A30" s="1" t="s">
         <v>149</v>
       </c>
@@ -11953,7 +11962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8">
       <c r="A31" s="1" t="s">
         <v>149</v>
       </c>
@@ -11979,7 +11988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8">
       <c r="A32" s="1" t="s">
         <v>149</v>
       </c>
@@ -12005,7 +12014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8">
       <c r="A33" s="1" t="s">
         <v>158</v>
       </c>
@@ -12031,7 +12040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8">
       <c r="A34" s="1" t="s">
         <v>158</v>
       </c>
@@ -12057,7 +12066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8">
       <c r="A35" s="1" t="s">
         <v>158</v>
       </c>
@@ -12083,7 +12092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8">
       <c r="A36" s="1" t="s">
         <v>158</v>
       </c>
@@ -12109,7 +12118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8">
       <c r="A37" s="1" t="s">
         <v>163</v>
       </c>
@@ -12135,7 +12144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8">
       <c r="A38" s="1" t="s">
         <v>163</v>
       </c>
@@ -12161,7 +12170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8">
       <c r="A39" s="1" t="s">
         <v>163</v>
       </c>
@@ -12187,7 +12196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8">
       <c r="A40" s="1" t="s">
         <v>163</v>
       </c>
@@ -12213,7 +12222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8">
       <c r="A41" s="1" t="s">
         <v>169</v>
       </c>
@@ -12239,7 +12248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8">
       <c r="A42" s="1" t="s">
         <v>187</v>
       </c>
@@ -12265,7 +12274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8">
       <c r="A43" s="1" t="s">
         <v>204</v>
       </c>
@@ -12291,7 +12300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8">
       <c r="A44" s="1" t="s">
         <v>221</v>
       </c>
@@ -12317,7 +12326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8">
       <c r="A45" s="1" t="s">
         <v>239</v>
       </c>
@@ -12343,7 +12352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8">
       <c r="A46" s="1" t="s">
         <v>257</v>
       </c>
@@ -12369,7 +12378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8">
       <c r="A47" s="1" t="s">
         <v>271</v>
       </c>
@@ -12395,7 +12404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8">
       <c r="A48" s="1" t="s">
         <v>271</v>
       </c>
@@ -12421,7 +12430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8">
       <c r="A49" s="1" t="s">
         <v>271</v>
       </c>
@@ -12447,7 +12456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8">
       <c r="A50" s="1" t="s">
         <v>271</v>
       </c>
@@ -12473,7 +12482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8">
       <c r="A51" s="1" t="s">
         <v>280</v>
       </c>
@@ -12499,7 +12508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8">
       <c r="A52" s="1" t="s">
         <v>280</v>
       </c>
@@ -12525,7 +12534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8">
       <c r="A53" s="1" t="s">
         <v>280</v>
       </c>
@@ -12551,7 +12560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8">
       <c r="A54" s="1" t="s">
         <v>280</v>
       </c>
@@ -12577,7 +12586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8">
       <c r="A55" s="1" t="s">
         <v>280</v>
       </c>
@@ -12603,7 +12612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8">
       <c r="A56" s="1" t="s">
         <v>286</v>
       </c>
@@ -12629,7 +12638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8">
       <c r="A57" s="1" t="s">
         <v>286</v>
       </c>
@@ -12655,7 +12664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8">
       <c r="A58" s="1" t="s">
         <v>286</v>
       </c>
@@ -12681,7 +12690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8">
       <c r="A59" s="1" t="s">
         <v>286</v>
       </c>
@@ -12707,7 +12716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8">
       <c r="A60" s="1" t="s">
         <v>291</v>
       </c>
@@ -12733,7 +12742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8">
       <c r="A61" s="1" t="s">
         <v>291</v>
       </c>
@@ -12759,7 +12768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8">
       <c r="A62" s="1" t="s">
         <v>291</v>
       </c>
@@ -12785,7 +12794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8">
       <c r="A63" s="1" t="s">
         <v>299</v>
       </c>
@@ -12811,7 +12820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8">
       <c r="A64" s="1" t="s">
         <v>299</v>
       </c>
@@ -12837,7 +12846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8">
       <c r="A65" s="1" t="s">
         <v>299</v>
       </c>
@@ -12863,7 +12872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8">
       <c r="A66" s="1" t="s">
         <v>304</v>
       </c>
@@ -12889,7 +12898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8">
       <c r="A67" s="1" t="s">
         <v>304</v>
       </c>
@@ -12915,7 +12924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8">
       <c r="A68" s="1" t="s">
         <v>304</v>
       </c>
@@ -12941,7 +12950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8">
       <c r="A69" s="1" t="s">
         <v>309</v>
       </c>
@@ -12967,7 +12976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8">
       <c r="A70" s="1" t="s">
         <v>309</v>
       </c>
@@ -12993,7 +13002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8">
       <c r="A71" s="1" t="s">
         <v>309</v>
       </c>
@@ -13019,7 +13028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8">
       <c r="A72" s="1" t="s">
         <v>309</v>
       </c>
@@ -13045,7 +13054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8">
       <c r="A73" s="1" t="s">
         <v>318</v>
       </c>
@@ -13071,7 +13080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8">
       <c r="A74" s="1" t="s">
         <v>318</v>
       </c>
@@ -13097,7 +13106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8">
       <c r="A75" s="1" t="s">
         <v>318</v>
       </c>
@@ -13123,7 +13132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8">
       <c r="A76" s="1" t="s">
         <v>318</v>
       </c>
@@ -13149,7 +13158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8">
       <c r="A77" s="1" t="s">
         <v>328</v>
       </c>
@@ -13175,7 +13184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8">
       <c r="A78" s="1" t="s">
         <v>346</v>
       </c>
@@ -13201,7 +13210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8">
       <c r="A79" s="1" t="s">
         <v>352</v>
       </c>
@@ -13227,7 +13236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8">
       <c r="A80" s="1" t="s">
         <v>358</v>
       </c>
@@ -13253,7 +13262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11">
       <c r="A81" s="1" t="s">
         <v>364</v>
       </c>
@@ -13279,7 +13288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11">
       <c r="A82" s="1" t="s">
         <v>370</v>
       </c>
@@ -13305,12 +13314,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11">
       <c r="A83" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B83" s="2">
-        <v>23301</v>
+      <c r="B83" s="3" t="s">
+        <v>438</v>
       </c>
       <c r="C83" s="1">
         <v>28800000</v>
@@ -13331,7 +13340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11">
       <c r="A84" s="1" t="s">
         <v>433</v>
       </c>
@@ -13357,7 +13366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11">
       <c r="K86" t="s">
         <v>436</v>
       </c>
@@ -13371,9 +13380,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -13399,7 +13408,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
@@ -13425,7 +13434,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
         <v>107</v>
       </c>
@@ -13451,7 +13460,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>115</v>
       </c>
@@ -13477,7 +13486,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
@@ -13503,7 +13512,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
         <v>128</v>
       </c>
@@ -13529,7 +13538,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
         <v>138</v>
       </c>
@@ -13555,7 +13564,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
         <v>144</v>
       </c>
@@ -13581,7 +13590,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
         <v>149</v>
       </c>
@@ -13607,7 +13616,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
         <v>158</v>
       </c>
@@ -13633,7 +13642,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="1" t="s">
         <v>163</v>
       </c>
@@ -13659,7 +13668,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8">
       <c r="A12" s="1" t="s">
         <v>168</v>
       </c>
@@ -13685,7 +13694,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8">
       <c r="A13" s="1" t="s">
         <v>169</v>
       </c>
@@ -13711,7 +13720,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="1" t="s">
         <v>187</v>
       </c>
@@ -13737,7 +13746,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8">
       <c r="A15" s="1" t="s">
         <v>204</v>
       </c>
@@ -13763,7 +13772,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8">
       <c r="A16" s="1" t="s">
         <v>221</v>
       </c>
@@ -13789,7 +13798,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="1" t="s">
         <v>239</v>
       </c>
@@ -13815,7 +13824,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="1" t="s">
         <v>257</v>
       </c>
@@ -13841,7 +13850,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
         <v>271</v>
       </c>
@@ -13867,7 +13876,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="1" t="s">
         <v>280</v>
       </c>
@@ -13893,7 +13902,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
         <v>286</v>
       </c>
@@ -13919,7 +13928,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="1" t="s">
         <v>291</v>
       </c>
@@ -13945,7 +13954,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8">
       <c r="A23" s="1" t="s">
         <v>299</v>
       </c>
@@ -13971,7 +13980,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8">
       <c r="A24" s="1" t="s">
         <v>304</v>
       </c>
@@ -13997,7 +14006,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8">
       <c r="A25" s="1" t="s">
         <v>309</v>
       </c>
@@ -14023,7 +14032,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8">
       <c r="A26" s="1" t="s">
         <v>318</v>
       </c>
@@ -14049,7 +14058,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8">
       <c r="A27" s="1" t="s">
         <v>328</v>
       </c>
@@ -14075,7 +14084,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8">
       <c r="A28" s="1" t="s">
         <v>346</v>
       </c>
@@ -14101,7 +14110,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8">
       <c r="A29" s="1" t="s">
         <v>352</v>
       </c>
@@ -14127,7 +14136,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8">
       <c r="A30" s="1" t="s">
         <v>358</v>
       </c>
@@ -14153,7 +14162,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8">
       <c r="A31" s="1" t="s">
         <v>364</v>
       </c>
@@ -14179,7 +14188,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8">
       <c r="A32" s="1" t="s">
         <v>370</v>
       </c>
@@ -14205,7 +14214,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8">
       <c r="A33" s="1" t="s">
         <v>377</v>
       </c>
@@ -14231,7 +14240,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8">
       <c r="A34" s="1" t="s">
         <v>378</v>
       </c>
@@ -14257,7 +14266,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8">
       <c r="A35" s="1" t="s">
         <v>379</v>
       </c>
@@ -14283,7 +14292,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8">
       <c r="A36" s="1" t="s">
         <v>380</v>
       </c>
@@ -14309,7 +14318,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8">
       <c r="A37" s="1" t="s">
         <v>381</v>
       </c>
@@ -14335,7 +14344,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8">
       <c r="A38" s="1" t="s">
         <v>382</v>
       </c>
@@ -14361,7 +14370,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8">
       <c r="A39" s="1" t="s">
         <v>383</v>
       </c>
@@ -14387,7 +14396,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8">
       <c r="A40" s="1" t="s">
         <v>384</v>
       </c>
@@ -14413,7 +14422,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8">
       <c r="A41" s="1" t="s">
         <v>385</v>
       </c>
@@ -14439,7 +14448,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8">
       <c r="A42" s="1" t="s">
         <v>386</v>
       </c>
@@ -14465,7 +14474,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8">
       <c r="A43" s="1" t="s">
         <v>387</v>
       </c>
@@ -14491,7 +14500,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8">
       <c r="A44" s="1" t="s">
         <v>388</v>
       </c>
@@ -14517,7 +14526,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8">
       <c r="A45" s="1" t="s">
         <v>389</v>
       </c>
@@ -14543,7 +14552,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8">
       <c r="A46" s="1" t="s">
         <v>390</v>
       </c>
@@ -14569,7 +14578,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8">
       <c r="A47" s="1" t="s">
         <v>391</v>
       </c>
@@ -14595,7 +14604,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8">
       <c r="A48" s="1" t="s">
         <v>392</v>
       </c>
@@ -14621,7 +14630,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8">
       <c r="A49" s="1" t="s">
         <v>393</v>
       </c>
@@ -14647,7 +14656,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8">
       <c r="A50" s="1" t="s">
         <v>394</v>
       </c>
@@ -14673,7 +14682,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8">
       <c r="A51" s="1" t="s">
         <v>395</v>
       </c>
@@ -14699,7 +14708,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8">
       <c r="A52" s="1" t="s">
         <v>396</v>
       </c>
@@ -14725,7 +14734,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8">
       <c r="A53" s="1" t="s">
         <v>427</v>
       </c>
@@ -14751,7 +14760,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8">
       <c r="A54" s="1" t="s">
         <v>428</v>
       </c>
@@ -14777,7 +14786,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8">
       <c r="A55" s="1" t="s">
         <v>429</v>
       </c>
@@ -14803,7 +14812,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8">
       <c r="A56" s="1" t="s">
         <v>430</v>
       </c>
@@ -14829,7 +14838,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8">
       <c r="A57" s="1" t="s">
         <v>431</v>
       </c>
@@ -14855,7 +14864,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8">
       <c r="A58" s="1" t="s">
         <v>432</v>
       </c>
@@ -14890,9 +14899,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>397</v>
       </c>
@@ -14915,7 +14924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>398</v>
       </c>
@@ -14938,7 +14947,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -14961,7 +14970,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="1">
         <v>51</v>
       </c>
@@ -14984,7 +14993,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="1">
         <v>101</v>
       </c>
@@ -15007,7 +15016,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" s="1">
         <v>151</v>
       </c>
@@ -15030,7 +15039,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" s="1">
         <v>201</v>
       </c>
@@ -15053,7 +15062,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" s="1">
         <v>251</v>
       </c>
@@ -15076,7 +15085,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9" s="1">
         <v>46</v>
       </c>

</xml_diff>